<commit_message>
Classify 4 previously confirmed rows as confirmed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017FBQtzqMjgKdgBTwMV3Uy9
</commit_message>
<xml_diff>
--- a/leads/Master_Leads_-_Best_600_verified.xlsx
+++ b/leads/Master_Leads_-_Best_600_verified.xlsx
@@ -851,7 +851,7 @@
           <t>+974 3013 4794</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>hello@mogobogo.qa</t>
         </is>
@@ -868,7 +868,11 @@
       </c>
       <c r="I5" s="6" t="n"/>
       <c r="J5" s="6" t="n"/>
-      <c r="K5" s="7" t="n"/>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>hello@mogobogo.qa</t>
+        </is>
+      </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
           <t>hello@mogobogo.qa</t>
@@ -881,12 +885,12 @@
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>Confirmed on their own site in the earlier check; domain matches site - kept</t>
+          <t>Confirmed on their own site in the earlier check; domain matches site</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Kept, unverified</t>
+          <t>Confirmed</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1058,7 @@
           <t>+974 6665 4472</t>
         </is>
       </c>
-      <c r="F8" s="10" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>info@marmarayistanbulrestaurant.com</t>
         </is>
@@ -1071,7 +1075,11 @@
       </c>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
-      <c r="K8" s="7" t="n"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>info@marmarayistanbulrestaurant.com</t>
+        </is>
+      </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
           <t>info@marmarayistanbulrestaurant.com</t>
@@ -1084,12 +1092,12 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>Confirmed on their own site in the earlier check; domain matches site - kept</t>
+          <t>Confirmed on their own site in the earlier check; domain matches site</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Kept, unverified</t>
+          <t>Confirmed</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1125,7 @@
           <t>+974 3004 7326</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>c.support@sabahwmasa.com</t>
         </is>
@@ -1138,7 +1146,11 @@
           <t>info@sabahwmasa.com</t>
         </is>
       </c>
-      <c r="K9" s="7" t="n"/>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>c.support@sabahwmasa.com</t>
+        </is>
+      </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
           <t>c.support@sabahwmasa.com</t>
@@ -1151,12 +1163,12 @@
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>Confirmed on their own site in the earlier check; domain matches site - kept</t>
+          <t>Confirmed on their own site in the earlier check; domain matches site</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Kept, unverified</t>
+          <t>Confirmed</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2184,7 @@
           <t>+974 5000 8852</t>
         </is>
       </c>
-      <c r="F24" s="10" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>sales@greydoha.qa</t>
         </is>
@@ -2189,7 +2201,11 @@
       </c>
       <c r="I24" s="6" t="n"/>
       <c r="J24" s="6" t="n"/>
-      <c r="K24" s="7" t="n"/>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>sales@greydoha.qa</t>
+        </is>
+      </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
           <t>sales@greydoha.qa</t>
@@ -2202,12 +2218,12 @@
       </c>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>Confirmed on their own site in the earlier check; domain matches site - kept</t>
+          <t>Confirmed on their own site in the earlier check; domain matches site</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Kept, unverified</t>
+          <t>Confirmed</t>
         </is>
       </c>
     </row>

</xml_diff>